<commit_message>
remove sdtm_mapping from crf
</commit_message>
<xml_diff>
--- a/project/crf/excel/cosmos_crf_model.xlsx
+++ b/project/crf/excel/cosmos_crf_model.xlsx
@@ -714,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -726,11 +726,6 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>sdtmVariables</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sdtmTargetMapping</t>
         </is>
       </c>
     </row>

</xml_diff>